<commit_message>
Actualizar planillas prestadores: dedup + categoria Centro Medico para honorarios medicos
</commit_message>
<xml_diff>
--- a/flujo_bancario/TABLERO_Resumen.xlsx
+++ b/flujo_bancario/TABLERO_Resumen.xlsx
@@ -448,7 +448,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -467,7 +467,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -486,26 +486,26 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>86596208.19000001</v>
+        <v>85359803.48000002</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>1236404.71</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -515,16 +515,16 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>1236404.71</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -543,7 +543,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -562,7 +562,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -581,7 +581,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -600,26 +600,26 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>85359803.48000002</v>
+        <v>84309803.48000002</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>1050000</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -629,16 +629,16 @@
         <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>1050000</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -657,26 +657,26 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>84309803.48000002</v>
+        <v>82982043.48000002</v>
       </c>
       <c r="C13" t="n">
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>1327760</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -686,35 +686,35 @@
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>1327760</v>
+        <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>82982043.48000002</v>
+        <v>75867964.53000002</v>
       </c>
       <c r="C15" t="n">
         <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>7114078.95</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -724,16 +724,16 @@
         <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>7114078.95</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -752,7 +752,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -771,7 +771,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -790,26 +790,26 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>75867964.53000002</v>
+        <v>-153105388.2</v>
       </c>
       <c r="C20" t="n">
         <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>228973352.73</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>71</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -819,16 +819,16 @@
         <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>228973352.73</v>
+        <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -847,26 +847,26 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>-153105388.2</v>
+        <v>-158105388.2</v>
       </c>
       <c r="C23" t="n">
         <v>0</v>
       </c>
       <c r="D23" t="n">
-        <v>0</v>
+        <v>5000000</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -876,16 +876,16 @@
         <v>0</v>
       </c>
       <c r="D24" t="n">
-        <v>5000000</v>
+        <v>0</v>
       </c>
       <c r="E24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -904,7 +904,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -923,7 +923,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -942,7 +942,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -961,26 +961,26 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>-158105388.2</v>
+        <v>-163105388.2</v>
       </c>
       <c r="C29" t="n">
         <v>0</v>
       </c>
       <c r="D29" t="n">
-        <v>0</v>
+        <v>5000000</v>
       </c>
       <c r="E29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -990,16 +990,16 @@
         <v>0</v>
       </c>
       <c r="D30" t="n">
-        <v>5000000</v>
+        <v>0</v>
       </c>
       <c r="E30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1018,7 +1018,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B32" t="n">

</xml_diff>

<commit_message>
actualizar y agregar comercial
</commit_message>
<xml_diff>
--- a/flujo_bancario/TABLERO_Resumen.xlsx
+++ b/flujo_bancario/TABLERO_Resumen.xlsx
@@ -448,17 +448,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-83261303.01999995</v>
+        <v>-89214378.09999995</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>5000000</v>
+        <v>5953075.08</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -467,17 +467,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-89214378.09999995</v>
+        <v>-89775712.55999994</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>5953075.08</v>
+        <v>561334.46</v>
       </c>
       <c r="E3" t="n">
         <v>1</v>
@@ -486,7 +486,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -496,16 +496,16 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>561334.46</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -524,26 +524,26 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-89775712.55999994</v>
+        <v>-94873168.03999995</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>5097455.48</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -553,35 +553,35 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>5097455.48</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-94873168.03999995</v>
+        <v>-99873168.03999995</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>5000000</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -591,16 +591,16 @@
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>5000000</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -619,7 +619,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -638,7 +638,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -657,7 +657,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -676,7 +676,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -695,7 +695,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -714,7 +714,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -733,26 +733,26 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-99873168.03999995</v>
+        <v>-100031434.6999999</v>
       </c>
       <c r="C17" t="n">
         <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>158266.66</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -762,35 +762,35 @@
         <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>158266.66</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>-100031434.6999999</v>
+        <v>-105031434.6999999</v>
       </c>
       <c r="C19" t="n">
         <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>5000000</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -800,45 +800,45 @@
         <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>5000000</v>
+        <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-105031434.6999999</v>
+        <v>-115767550.3599999</v>
       </c>
       <c r="C21" t="n">
         <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>10736115.66</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>-115767550.3599999</v>
+        <v>-120767550.3599999</v>
       </c>
       <c r="C22" t="n">
         <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>10736115.66</v>
+        <v>5000000</v>
       </c>
       <c r="E22" t="n">
         <v>1</v>
@@ -847,7 +847,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -857,16 +857,16 @@
         <v>0</v>
       </c>
       <c r="D23" t="n">
-        <v>5000000</v>
+        <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -885,7 +885,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -904,7 +904,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -923,26 +923,26 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>-120767550.3599999</v>
+        <v>-334894558.92</v>
       </c>
       <c r="C27" t="n">
         <v>0</v>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>214127008.56</v>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -952,16 +952,16 @@
         <v>0</v>
       </c>
       <c r="D28" t="n">
-        <v>214127008.56</v>
+        <v>0</v>
       </c>
       <c r="E28" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -980,45 +980,45 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>-334894558.92</v>
+        <v>-339894558.92</v>
       </c>
       <c r="C30" t="n">
         <v>0</v>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>5000000</v>
       </c>
       <c r="E30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>-339894558.92</v>
+        <v>-343792943.2499999</v>
       </c>
       <c r="C31" t="n">
         <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>5000000</v>
+        <v>3898384.33</v>
       </c>
       <c r="E31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1028,10 +1028,10 @@
         <v>0</v>
       </c>
       <c r="D32" t="n">
-        <v>3898384.33</v>
+        <v>0</v>
       </c>
       <c r="E32" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>